<commit_message>
feat: detail_search_extractor.py 추가 — 계정별원장 직접 추출 (웹 UI 우회)
host1_상세검색_시나리오 task_list 시트를 읽어 계정별원장 xlsx에서
직접 데이터를 추출한다. graphy처럼 웹 UI 상세검색이 열 명칭 차이로
동작하지 않는 경우의 대안. host1_상세검색_시나리오 시트가 없는 회사는
무시하고 정상 종료하므로 다른 회사에 영향 없음.
run.bat extract/all 단계에 [2/3], [2/5] 단계로 자동 포함.

graphy 결과: 특수관계자거래(1건) / 유형자산취득거래(7건) /
             은행조회서완전성(88건) / 리스거래완전성(5230건)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/graphy/results/graphy_20260512_유형자산취득거래.xlsx
+++ b/graphy/results/graphy_20260512_유형자산취득거래.xlsx
@@ -1,29 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
-  <calcPr calcId="171027"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
+  <sheets>
+    <sheet name="유형자산취득거래" sheetId="1" state="visible" r:id="rId1"/>
+  </sheets>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <color theme="1"/>
-      <family val="2"/>
+      <sz val="11"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -38,22 +56,85 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -132,7 +213,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -167,7 +247,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -202,16 +281,20 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:shade val="100000"/>
-                <a:satMod val="350000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -333,46 +416,274 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:spDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="3">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </a:style>
-    </a:spDef>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
 </a:theme>
+</file>
+
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>계정과목</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>날짜</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>적요란</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>거래처명</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>사업자등록번호</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>건물</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>에이스가산포휴 611호 B027</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="2" t="n">
+        <v>732889449</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>건물</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>에이스가산포휴 612호 B028</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" s="2" t="n">
+        <v>628042723</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>건물</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025-10-31</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>가산포휴 611~612 인테리어 비용 B029</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>디자인살랑</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>562-09-03129</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>10900000</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>기계장치</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2025-11-30</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>코맥스 기계장치 인식 E069</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>(주)코맥스</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>452-87-00556</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>1636364</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>기계장치</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>코맥스 기계장치 인식 E070</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>(주)코맥스</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>452-87-00556</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>3090909</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2025-03-05</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>THC2 Door 금형비 잔금 지급 요청의 건_트라이텍 공구와기구 대체 R112</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>주식회사 트라이텍</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>633-88-01559</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>27200000</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>공구와기구</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2025-06-30</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>6월 사무용품 유형자산 전환 R113</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" s="2" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>